<commit_message>
Added customized holiday method and Removed not so important features
</commit_message>
<xml_diff>
--- a/Holiday_Off_Time_Info.xlsx
+++ b/Holiday_Off_Time_Info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devan\Desktop\SAR_Work\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78A45A9F-84F5-40F1-A8C8-9022D8212107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FCD5BD6-6B16-49F3-A7E6-3A3B4600ABF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,10 +51,10 @@
     <t>EndTime</t>
   </si>
   <si>
-    <t>23/02/2026, 07:00:00</t>
-  </si>
-  <si>
-    <t>24/02/2026, 06:00:00</t>
+    <t>23/02/2026, 12:00:00</t>
+  </si>
+  <si>
+    <t>23/02/2026, 16:00:00</t>
   </si>
 </sst>
 </file>

</xml_diff>